<commit_message>
Mark GPT-4o as public (🔴 → 🟢)
The sheet had GPT-4o as 🔴 (held in the lab, never released), so the
constellation drew it as a hollow "unreleased" dot. OpenAI's launch post
says it rolled out in ChatGPT, free tier included, and the API on
2024-05-13. The note on the row records the change and its source.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155Jn554N4wF8sUPizjhCxA
</commit_message>
<xml_diff>
--- a/Pruned AI Models_Table.xlsx
+++ b/Pruned AI Models_Table.xlsx
@@ -24686,7 +24686,7 @@
       </c>
       <c r="O343" s="30" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="P343" s="30" t="inlineStr">
@@ -24706,7 +24706,7 @@
       </c>
       <c r="S343" s="33" t="inlineStr">
         <is>
-          <t>gpt-4o-2024-05-13 no longer easily available, so hidden in the Model Table rankings. Omnimodel. ‘[GPT-4o is] likely an early checkpoint of GPT-5’. https://twitter.com/drjimfan/status/1790089671365767313 ELO: https://twitter.com/LiamFedus/status/1790064963966370209 Demo: https://youtu.be/DQacCB9tDaw</t>
+          <t>gpt-4o-2024-05-13 no longer easily available, so hidden in the Model Table rankings. Omnimodel. ‘[GPT-4o is] likely an early checkpoint of GPT-5’. https://twitter.com/drjimfan/status/1790089671365767313 ELO: https://twitter.com/LiamFedus/status/1790064963966370209 Demo: https://youtu.be/DQacCB9tDaw Public? changed from 🔴 to 🟢 on 2026-09-27: OpenAI's launch post says GPT-4o's text and image capabilities started rolling out in ChatGPT, including the free tier, and in the API on 2024-05-13. Source: https://openai.com/index/hello-gpt-4o/.</t>
         </is>
       </c>
       <c r="T343" s="31" t="n">

</xml_diff>